<commit_message>
added testng,rename the file name and modify keyword
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -1,22 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hp\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F5B33C3C-4482-489B-ACE8-AA01F4C2F787}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{FEB9E3EC-3D2F-42D0-9DEB-F8823D610FEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C57D25BF-7E00-4FA5-B23A-EA3980E632DD}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{C57D25BF-7E00-4FA5-B23A-EA3980E632DD}"/>
   </bookViews>
   <sheets>
     <sheet name="lip_brands" sheetId="1" r:id="rId1"/>
     <sheet name="validPincodes" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1:M13"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -500,92 +497,92 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4DF986B-CB36-4ED3-BEFB-C75FD0A5EBDC}">
   <dimension ref="A1:A17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.21875" customWidth="1"/>
+    <col min="1" max="1" width="14.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>11</v>
       </c>
@@ -598,72 +595,72 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4631B343-F4C7-4538-8307-2C0FD8998D4C}">
   <dimension ref="A1:A13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="27.21875" customWidth="1"/>
+    <col min="1" max="1" width="27.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:1" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>28</v>
       </c>
@@ -671,4 +668,13 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9F98709-7E98-4879-A5BA-9DEF51DCE820}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>